<commit_message>
Discretização para uma dimensão
</commit_message>
<xml_diff>
--- a/saida.xlsx
+++ b/saida.xlsx
@@ -437,607 +437,607 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0</v>
+        <v>2.999999999999979</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.1</v>
+        <v>2.98501249583412</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0.2</v>
+        <v>2.940199733523704</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0.3</v>
+        <v>2.866009467376756</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0.4</v>
+        <v>2.763182982008635</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0.5</v>
+        <v>2.63274768567107</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>0.6000000000000001</v>
+        <v>2.47600684472908</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>0.7000000000000001</v>
+        <v>2.294526561853487</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>0.8</v>
+        <v>2.090120128041492</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0.9</v>
+        <v>1.864829904812004</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>1</v>
+        <v>1.620906917604425</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>0.1695018627821161</v>
+        <v>3.099833416646807</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>0.2512384585136417</v>
+        <v>3.136006745950143</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>0.3418060975042272</v>
+        <v>3.111493121730769</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>0.4370846409905623</v>
+        <v>3.046498884437139</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>0.5362545304265818</v>
+        <v>2.947904633097211</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>0.636299640234486</v>
+        <v>2.818751418855172</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>0.7362545303892744</v>
+        <v>2.660817742999205</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>0.8370846409237261</v>
+        <v>2.475160473516042</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>0.9418060974071489</v>
+        <v>2.26155758502611</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>1.051238458392336</v>
+        <v>2.015911999461014</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>1.169501862661777</v>
+        <v>1.720740334251253</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>0.3030569697280784</v>
+        <v>3.298502747441828</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>0.3859494876467936</v>
+        <v>3.315835050391654</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>0.470327828222519</v>
+        <v>3.291859751391772</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>0.5667571762674489</v>
+        <v>3.229921725939766</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>0.662590944305359</v>
+        <v>3.13354649709152</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>0.7639983697156553</v>
+        <v>3.005201142155622</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>0.862590944219698</v>
+        <v>2.846585336798006</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>0.9667571760956716</v>
+        <v>2.658788395374387</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>1.070327828012614</v>
+        <v>2.442131325659344</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>1.185949487364549</v>
+        <v>2.195869212616147</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>1.303056969447032</v>
+        <v>1.919409665046275</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>0.4313608353967657</v>
+        <v>3.494189537456339</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>0.513597332940404</v>
+        <v>3.503136891008788</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>0.5956520880199428</v>
+        <v>3.476798015318525</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>0.6912030765927899</v>
+        <v>3.415130222714767</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>0.7857015443076433</v>
+        <v>3.319534277599846</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>0.8869201881648684</v>
+        <v>3.191601287702682</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>0.9857015441253146</v>
+        <v>3.032781802140251</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>1.091203076240114</v>
+        <v>2.844340031520182</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>1.19565208758287</v>
+        <v>2.627420133298109</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>1.313597332390145</v>
+        <v>2.383391833649939</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>1.431360834848366</v>
+        <v>2.115096455060785</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>0.5545777403125538</v>
+        <v>3.684938548970044</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>0.6372276232389071</v>
+        <v>3.689951074142426</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>0.7218504318059769</v>
+        <v>3.661732350604547</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>0.8126637021294737</v>
+        <v>3.599672513523877</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>0.9070153987984955</v>
+        <v>3.504291627152698</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>1.005570046145002</v>
+        <v>3.376624552599313</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>1.107015398434671</v>
+        <v>3.217905136178444</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>1.21266370146264</v>
+        <v>3.029490758082487</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>1.32185043093767</v>
+        <v>2.812985802954772</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>1.437227622251725</v>
+        <v>2.57060980556346</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>1.554577739326763</v>
+        <v>2.305845466574434</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>0.6751042859404092</v>
+        <v>3.868843880912904</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>0.7562661032628687</v>
+        <v>3.87234333108036</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>0.839633885298522</v>
+        <v>3.843294625451738</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>0.92794427257235</v>
+        <v>3.78106055907442</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>1.019474194655182</v>
+        <v>3.685886501041581</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>1.114645257048027</v>
+        <v>3.558555584045963</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>1.219474194019294</v>
+        <v>3.400146981241495</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>1.327944271420143</v>
+        <v>3.211972341114296</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>1.439633883828165</v>
+        <v>2.995710904927975</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>1.556266101634527</v>
+        <v>2.753765265170749</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>1.675104284305864</v>
+        <v>2.489750798517309</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>0.7940691611588824</v>
+        <v>4.044068011999181</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>0.870955377161687</v>
+        <v>4.047830424804852</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>0.9512247660692386</v>
+        <v>4.019028856288735</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>1.0377275881769</v>
+        <v>3.957113041002394</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>1.124454824511941</v>
+        <v>3.862389359055929</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>1.226182036767627</v>
+        <v>3.735619614345694</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>1.324454823447533</v>
+        <v>3.577778410570543</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>1.43772758625687</v>
+        <v>3.389981084917388</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>1.551224763719637</v>
+        <v>3.173608727696119</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>1.67095537463433</v>
+        <v>2.93073878196197</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>1.794069158573745</v>
+        <v>2.664974929603622</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>0.8970905046251362</v>
+        <v>4.208860160632677</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>0.9792750785131049</v>
+        <v>4.214725023468602</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>1.054652519008459</v>
+        <v>4.187161580177905</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>1.144039901544231</v>
+        <v>4.12599602814865</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>1.23692677790156</v>
+        <v>4.031987958742284</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>1.340086445750239</v>
+        <v>3.906109184232218</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>1.436926776108479</v>
+        <v>3.749288328112764</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>1.544039898363385</v>
+        <v>3.562303867348663</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>1.654652515411276</v>
+        <v>3.345790783406585</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>1.779275074866566</v>
+        <v>3.100652590301356</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>1.89709050071915</v>
+        <v>2.829767078237121</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>1.01175372348312</v>
+        <v>4.361573778137292</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>1.095368475103877</v>
+        <v>4.372302161481966</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>1.178296952889788</v>
+        <v>4.346592924022051</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>1.267728977116833</v>
+        <v>4.286157426293876</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>1.361957497904592</v>
+        <v>4.192920778640273</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>1.461006219399807</v>
+        <v>4.068309035809878</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>1.561957495857589</v>
+        <v>3.913298340153593</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>1.667728973587356</v>
+        <v>3.72830803671753</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>1.778296948652662</v>
+        <v>3.512797417950622</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>1.895368470519823</v>
+        <v>3.264771200824022</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>2.011753718513565</v>
+        <v>2.982480695741577</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>1.134734311014382</v>
+        <v>4.500683000526967</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
-        <v>1.215503262816099</v>
+        <v>4.522111478379418</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
-        <v>1.299074784237001</v>
+        <v>4.496989418178627</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
-        <v>1.388847323775439</v>
+        <v>4.436099433241835</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
-        <v>1.483518870930829</v>
+        <v>4.343236382039783</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
-        <v>1.581955764015214</v>
+        <v>4.220220453361415</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
-        <v>1.683518868478894</v>
+        <v>4.068168808160931</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
-        <v>1.78884731965917</v>
+        <v>3.887529206826195</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
-        <v>1.899074779318924</v>
+        <v>3.677061957944052</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
-        <v>2.015503257426972</v>
+        <v>3.430152280151807</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
-        <v>2.134734305055784</v>
+        <v>3.121589918131465</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
-        <v>1.234734311014382</v>
+        <v>4.682941969615854</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
-        <v>1.334734311014382</v>
+        <v>4.672950300171904</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
-        <v>1.416349713185045</v>
+        <v>4.638079290576299</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="n">
-        <v>1.506657005838492</v>
+        <v>4.573681525708298</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
-        <v>1.60202014260554</v>
+        <v>4.480400446747162</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="n">
-        <v>1.700409384073648</v>
+        <v>4.359168087399456</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="n">
-        <v>1.802020139392174</v>
+        <v>4.211195761325488</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="n">
-        <v>1.906657000805095</v>
+        <v>4.037961959094374</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
-        <v>2.016349707591686</v>
+        <v>3.841197575594527</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
-        <v>2.134734305055784</v>
+        <v>3.6228686155043</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
-        <v>2.234734305055781</v>
+        <v>3.385156549622764</v>
       </c>
     </row>
   </sheetData>

</xml_diff>